<commit_message>
04-04-2026 need to fix tax amount in db
</commit_message>
<xml_diff>
--- a/Roles&permission.xlsx
+++ b/Roles&permission.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="58">
   <si>
     <t>Role</t>
   </si>
@@ -186,6 +186,18 @@
   </si>
   <si>
     <t>Hide Admin side</t>
+  </si>
+  <si>
+    <t>roles</t>
+  </si>
+  <si>
+    <t>manage</t>
+  </si>
+  <si>
+    <t>assign_roles</t>
+  </si>
+  <si>
+    <t>assign</t>
   </si>
 </sst>
 </file>
@@ -510,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -857,6 +869,37 @@
         <v>5</v>
       </c>
     </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>54</v>
+      </c>
+      <c r="B74" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>56</v>
+      </c>
+      <c r="B78" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="261" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>

</xml_diff>